<commit_message>
Référentiel unique des listes apprenant : formulaires, import, sélecteur, dispositifs et modèle Excel générés depuis src/lib/referentiels.ts (npm run modele) + test anti-divergence
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/modeles/modele-apprenants.xlsx
+++ b/docs/modeles/modele-apprenants.xlsx
@@ -468,11 +468,11 @@
     <col width="26" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
     <col width="22" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
@@ -3203,13 +3203,13 @@
       <formula1>"femme,homme,autre"</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur invalide" error="Choisissez une valeur de la liste (ou laissez vide)." type="list">
-      <formula1>"Demandeur d'emploi,RSA,Salarié,Scolaire,Étudiant,Inactif"</formula1>
+      <formula1>"Demandeur d'emploi,RSA,Salarié,Scolaire / étudiant,Inactif / autre"</formula1>
     </dataValidation>
     <dataValidation sqref="M2:M500 N2:N500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur invalide" error="Choisissez une valeur de la liste (ou laissez vide)." type="list">
       <formula1>"oui,non"</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur invalide" error="Choisissez une valeur de la liste (ou laissez vide)." type="list">
-      <formula1>"Jamais scolarisé,Primaire,Collège,Lycée,Supérieur"</formula1>
+      <formula1>"Jamais scolarisé,Primaire,Secondaire,Supérieur"</formula1>
     </dataValidation>
     <dataValidation sqref="P2:P500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur invalide" error="Choisissez une valeur de la liste (ou laissez vide)." type="list">
       <formula1>"France Travail,Mission locale,CCAS,Spontané,Association partenaire,Autre"</formula1>
@@ -3228,7 +3228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -3242,40 +3242,40 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr"/>
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Généré automatiquement depuis le référentiel de l'application : les menus déroulants sont IDENTIQUES à ceux de l'ERP.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>1. Remplissez la feuille « Apprenants » : une ligne par personne. Seuls Prénom et Nom sont obligatoires.</t>
-        </is>
-      </c>
+      <c r="A3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>2. Supprimez les 2 lignes d'exemple (en vert pâle) avant l'import.</t>
+          <t>1. Remplissez la feuille « Apprenants » : une ligne par personne. Seuls Prénom et Nom sont obligatoires.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>3. Dans l'ERP : Apprenants → « Importer une liste » → « Choisir un fichier Excel » → sélectionnez ce fichier.</t>
+          <t>2. Supprimez les 2 lignes d'exemple (en vert pâle).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (Le copier-coller des lignes fonctionne aussi.)</t>
+          <t>3. Déposez ce fichier dans le dossier Drive partagé « Apprenant ERPPEF » : les nouvelles lignes sont importées chaque nuit (ou bouton « Synchroniser le Drive »).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>4. Vérifiez l'aperçu, choisissez éventuellement un groupe d'inscription, importez.</t>
+          <t xml:space="preserve">   Autre voie : ERP → Apprenants → « Importer une liste » → « Choisir un fichier Excel ».</t>
         </is>
       </c>
     </row>
@@ -3292,42 +3292,35 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>• Naissance au format JJ/MM/AAAA (la colonne est en texte : tapez 12/05/1988 tel quel).</t>
+          <t>• Naissance au format JJ/MM/AAAA (colonne en texte : tapez 12/05/1988 tel quel).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>• Niveau : laissez VIDE si inconnu — un test de positionnement sera généré automatiquement pour la personne.</t>
+          <t>• Niveau : laissez VIDE si inconnu — un test de positionnement sera généré automatiquement.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>• Les menus déroulants (Niveau, Sexe, Situation, QPV, RQTH, Scolarisation, Prescripteur, Quartier) évitent les fautes de frappe.</t>
+          <t>• Quartier : uniquement pour les résidents de Saint-Ouen.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>• Quartier : uniquement pour les résidents de Saint-Ouen.</t>
+          <t>• La typologie alimente directement vos bilans financeurs : plus c'est rempli, mieux c'est.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>• La typologie (naissance, sexe, commune, QPV…) alimente directement vos bilans financeurs : plus c'est rempli, mieux c'est.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>• Maximum 200 lignes par import (faites plusieurs imports au-delà).</t>
+          <t>• Maximum 200 lignes par import manuel (la synchronisation Drive n'a pas cette limite).</t>
         </is>
       </c>
     </row>

</xml_diff>